<commit_message>
Export FO 02-03: volver al formato del formulario, colores y cierre
Numeros con el formato contable (guion para el cero) y fechas dd/mm/yyyy en las tablas; la celda del periodo sigue en AAAA-MM-DD. Importes cruzados en amarillo y debitos del banco pendientes en rosado. El cierre pasa a Saldo Ajustado / Saldo segun Extracto con la formula =F(ajustado)-F(extracto).
</commit_message>
<xml_diff>
--- a/FO_02-03_DEMO.xlsx
+++ b/FO_02-03_DEMO.xlsx
@@ -17,9 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -40,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -50,6 +51,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD5A6BD"/>
       </patternFill>
     </fill>
   </fills>
@@ -136,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -171,18 +182,24 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -705,23 +722,23 @@
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr"/>
-      <c r="D10" s="16" t="n">
+      <c r="D10" s="20" t="n">
         <v>1250000</v>
       </c>
-      <c r="E10" s="16" t="n">
+      <c r="E10" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="16">
         <f>F9+D10-E10</f>
         <v/>
       </c>
-      <c r="G10" s="20" t="inlineStr">
+      <c r="G10" s="21" t="inlineStr">
         <is>
           <t>Factura A 1001 - Cliente Norte</t>
         </is>
       </c>
-      <c r="H10" s="20" t="inlineStr"/>
-      <c r="I10" s="20" t="inlineStr"/>
+      <c r="H10" s="21" t="inlineStr"/>
+      <c r="I10" s="21" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="18" t="n">
@@ -733,23 +750,23 @@
         </is>
       </c>
       <c r="C11" s="19" t="inlineStr"/>
-      <c r="D11" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="16" t="n">
+      <c r="D11" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="20" t="n">
         <v>1250000</v>
       </c>
       <c r="F11" s="16">
         <f>F10+D11-E11</f>
         <v/>
       </c>
-      <c r="G11" s="20" t="inlineStr">
+      <c r="G11" s="21" t="inlineStr">
         <is>
           <t>Cobro factura A 1001</t>
         </is>
       </c>
-      <c r="H11" s="20" t="inlineStr"/>
-      <c r="I11" s="20" t="inlineStr"/>
+      <c r="H11" s="21" t="inlineStr"/>
+      <c r="I11" s="21" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="18" t="n">
@@ -761,23 +778,23 @@
         </is>
       </c>
       <c r="C12" s="19" t="inlineStr"/>
-      <c r="D12" s="16" t="n">
+      <c r="D12" s="20" t="n">
         <v>845000.5</v>
       </c>
-      <c r="E12" s="16" t="n">
+      <c r="E12" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="16">
         <f>F11+D12-E12</f>
         <v/>
       </c>
-      <c r="G12" s="20" t="inlineStr">
+      <c r="G12" s="21" t="inlineStr">
         <is>
           <t>Factura A 1002 - Cliente Sur</t>
         </is>
       </c>
-      <c r="H12" s="20" t="inlineStr"/>
-      <c r="I12" s="20" t="inlineStr"/>
+      <c r="H12" s="21" t="inlineStr"/>
+      <c r="I12" s="21" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="18" t="n">
@@ -789,23 +806,23 @@
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr"/>
-      <c r="D13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="16" t="n">
+      <c r="D13" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="20" t="n">
         <v>320000</v>
       </c>
       <c r="F13" s="16">
         <f>F12+D13-E13</f>
         <v/>
       </c>
-      <c r="G13" s="20" t="inlineStr">
+      <c r="G13" s="21" t="inlineStr">
         <is>
           <t>Pago proveedor Logistica SRL</t>
         </is>
       </c>
-      <c r="H13" s="20" t="inlineStr"/>
-      <c r="I13" s="20" t="inlineStr"/>
+      <c r="H13" s="21" t="inlineStr"/>
+      <c r="I13" s="21" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="18" t="n">
@@ -817,23 +834,23 @@
         </is>
       </c>
       <c r="C14" s="19" t="inlineStr"/>
-      <c r="D14" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="16" t="n">
+      <c r="D14" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="20" t="n">
         <v>180000</v>
       </c>
       <c r="F14" s="16">
         <f>F13+D14-E14</f>
         <v/>
       </c>
-      <c r="G14" s="20" t="inlineStr">
+      <c r="G14" s="21" t="inlineStr">
         <is>
           <t>Honorarios contables</t>
         </is>
       </c>
-      <c r="H14" s="20" t="inlineStr"/>
-      <c r="I14" s="20" t="inlineStr"/>
+      <c r="H14" s="21" t="inlineStr"/>
+      <c r="I14" s="21" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="18" t="n">
@@ -845,23 +862,23 @@
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr"/>
-      <c r="D15" s="16" t="n">
+      <c r="D15" s="20" t="n">
         <v>15500.75</v>
       </c>
-      <c r="E15" s="16" t="n">
+      <c r="E15" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="16">
         <f>F14+D15-E15</f>
         <v/>
       </c>
-      <c r="G15" s="20" t="inlineStr">
+      <c r="G15" s="21" t="inlineStr">
         <is>
           <t>Comisiones bancarias</t>
         </is>
       </c>
-      <c r="H15" s="20" t="inlineStr"/>
-      <c r="I15" s="20" t="inlineStr"/>
+      <c r="H15" s="21" t="inlineStr"/>
+      <c r="I15" s="21" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="18" t="n">
@@ -873,23 +890,23 @@
         </is>
       </c>
       <c r="C16" s="19" t="inlineStr"/>
-      <c r="D16" s="16" t="n">
+      <c r="D16" s="20" t="n">
         <v>530000</v>
       </c>
-      <c r="E16" s="16" t="n">
+      <c r="E16" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="16">
         <f>F15+D16-E16</f>
         <v/>
       </c>
-      <c r="G16" s="20" t="inlineStr">
+      <c r="G16" s="21" t="inlineStr">
         <is>
           <t>Factura A 1003 - Cliente Centro</t>
         </is>
       </c>
-      <c r="H16" s="20" t="inlineStr"/>
-      <c r="I16" s="20" t="inlineStr"/>
+      <c r="H16" s="21" t="inlineStr"/>
+      <c r="I16" s="21" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="18" t="n">
@@ -901,23 +918,23 @@
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr"/>
-      <c r="D17" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="16" t="n">
+      <c r="D17" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="20" t="n">
         <v>96000</v>
       </c>
       <c r="F17" s="16">
         <f>F16+D17-E17</f>
         <v/>
       </c>
-      <c r="G17" s="20" t="inlineStr">
+      <c r="G17" s="21" t="inlineStr">
         <is>
           <t>Transferencia seguro</t>
         </is>
       </c>
-      <c r="H17" s="20" t="inlineStr"/>
-      <c r="I17" s="20" t="inlineStr"/>
+      <c r="H17" s="21" t="inlineStr"/>
+      <c r="I17" s="21" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="18" t="n">
@@ -929,23 +946,23 @@
         </is>
       </c>
       <c r="C18" s="19" t="inlineStr"/>
-      <c r="D18" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="16" t="n">
+      <c r="D18" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="20" t="n">
         <v>845000.5</v>
       </c>
       <c r="F18" s="16">
         <f>F17+D18-E18</f>
         <v/>
       </c>
-      <c r="G18" s="20" t="inlineStr">
+      <c r="G18" s="21" t="inlineStr">
         <is>
           <t>Cobro factura A 1002</t>
         </is>
       </c>
-      <c r="H18" s="20" t="inlineStr"/>
-      <c r="I18" s="20" t="inlineStr"/>
+      <c r="H18" s="21" t="inlineStr"/>
+      <c r="I18" s="21" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="18" t="n">
@@ -957,23 +974,23 @@
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr"/>
-      <c r="D19" s="16" t="n">
+      <c r="D19" s="20" t="n">
         <v>410000</v>
       </c>
-      <c r="E19" s="16" t="n">
+      <c r="E19" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="16">
         <f>F18+D19-E19</f>
         <v/>
       </c>
-      <c r="G19" s="20" t="inlineStr">
+      <c r="G19" s="21" t="inlineStr">
         <is>
           <t>Factura A 1004 - Cliente Norte</t>
         </is>
       </c>
-      <c r="H19" s="20" t="inlineStr"/>
-      <c r="I19" s="20" t="inlineStr"/>
+      <c r="H19" s="21" t="inlineStr"/>
+      <c r="I19" s="21" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="18" t="n">
@@ -985,23 +1002,23 @@
         </is>
       </c>
       <c r="C20" s="19" t="inlineStr"/>
-      <c r="D20" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="16" t="n">
+      <c r="D20" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="20" t="n">
         <v>250000</v>
       </c>
       <c r="F20" s="16">
         <f>F19+D20-E20</f>
         <v/>
       </c>
-      <c r="G20" s="20" t="inlineStr">
+      <c r="G20" s="21" t="inlineStr">
         <is>
           <t>Pago alquiler oficina</t>
         </is>
       </c>
-      <c r="H20" s="20" t="inlineStr"/>
-      <c r="I20" s="20" t="inlineStr"/>
+      <c r="H20" s="21" t="inlineStr"/>
+      <c r="I20" s="21" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="18" t="n">
@@ -1013,23 +1030,23 @@
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr"/>
-      <c r="D21" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="16" t="n">
+      <c r="D21" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="20" t="n">
         <v>3200.25</v>
       </c>
       <c r="F21" s="16">
         <f>F20+D21-E21</f>
         <v/>
       </c>
-      <c r="G21" s="20" t="inlineStr">
+      <c r="G21" s="21" t="inlineStr">
         <is>
           <t>Intereses ganados</t>
         </is>
       </c>
-      <c r="H21" s="20" t="inlineStr"/>
-      <c r="I21" s="20" t="inlineStr"/>
+      <c r="H21" s="21" t="inlineStr"/>
+      <c r="I21" s="21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="18" t="n">
@@ -1041,23 +1058,23 @@
         </is>
       </c>
       <c r="C22" s="19" t="inlineStr"/>
-      <c r="D22" s="16" t="n">
+      <c r="D22" s="20" t="n">
         <v>275000</v>
       </c>
-      <c r="E22" s="16" t="n">
+      <c r="E22" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="16">
         <f>F21+D22-E22</f>
         <v/>
       </c>
-      <c r="G22" s="20" t="inlineStr">
+      <c r="G22" s="21" t="inlineStr">
         <is>
           <t>Factura A 1005 - Cliente Sur</t>
         </is>
       </c>
-      <c r="H22" s="20" t="inlineStr"/>
-      <c r="I22" s="20" t="inlineStr"/>
+      <c r="H22" s="21" t="inlineStr"/>
+      <c r="I22" s="21" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="18" t="n">
@@ -1069,23 +1086,23 @@
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr"/>
-      <c r="D23" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="16" t="n">
+      <c r="D23" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="20" t="n">
         <v>198000</v>
       </c>
       <c r="F23" s="16">
         <f>F22+D23-E23</f>
         <v/>
       </c>
-      <c r="G23" s="20" t="inlineStr">
+      <c r="G23" s="21" t="inlineStr">
         <is>
           <t>Pago proveedor Insumos SA</t>
         </is>
       </c>
-      <c r="H23" s="20" t="inlineStr"/>
-      <c r="I23" s="20" t="inlineStr"/>
+      <c r="H23" s="21" t="inlineStr"/>
+      <c r="I23" s="21" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="18" t="n">
@@ -1107,13 +1124,13 @@
         <f>F23+D24-E24</f>
         <v/>
       </c>
-      <c r="G24" s="20" t="inlineStr">
+      <c r="G24" s="21" t="inlineStr">
         <is>
           <t>Cobro factura A 1003</t>
         </is>
       </c>
-      <c r="H24" s="20" t="inlineStr"/>
-      <c r="I24" s="20" t="inlineStr"/>
+      <c r="H24" s="21" t="inlineStr"/>
+      <c r="I24" s="21" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="17" t="inlineStr">
@@ -1170,26 +1187,26 @@
       </c>
       <c r="B28" s="19" t="inlineStr">
         <is>
-          <t>OP-0003-00000006</t>
+          <t>REC-0002-00000003</t>
         </is>
       </c>
       <c r="C28" s="19" t="inlineStr"/>
       <c r="D28" s="16" t="n">
-        <v>145000</v>
+        <v>0</v>
       </c>
       <c r="E28" s="16" t="n">
-        <v>0</v>
+        <v>530000</v>
       </c>
       <c r="F28" s="16">
         <f>D28-E28</f>
         <v/>
       </c>
-      <c r="G28" s="20" t="inlineStr">
-        <is>
-          <t>Cheque propio diferido</t>
-        </is>
-      </c>
-      <c r="H28" s="20" t="inlineStr"/>
+      <c r="G28" s="21" t="inlineStr">
+        <is>
+          <t>Cobro factura A 1003</t>
+        </is>
+      </c>
+      <c r="H28" s="21" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="18" t="n">
@@ -1211,12 +1228,12 @@
         <f>F28+D29-E29</f>
         <v/>
       </c>
-      <c r="G29" s="20" t="inlineStr">
+      <c r="G29" s="21" t="inlineStr">
         <is>
           <t>Factura A 1006 - pendiente de cobro</t>
         </is>
       </c>
-      <c r="H29" s="20" t="inlineStr"/>
+      <c r="H29" s="21" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
@@ -1282,9 +1299,9 @@
         <f>D33-E33</f>
         <v/>
       </c>
-      <c r="G33" s="20" t="inlineStr">
-        <is>
-          <t>Impuesto ley 25413 debito</t>
+      <c r="G33" s="21" t="inlineStr">
+        <is>
+          <t>IMPUESTO LEY 25413</t>
         </is>
       </c>
     </row>
@@ -1308,9 +1325,9 @@
         <f>F33+D34-E34</f>
         <v/>
       </c>
-      <c r="G34" s="20" t="inlineStr">
-        <is>
-          <t>Comision mantenimiento cuenta</t>
+      <c r="G34" s="21" t="inlineStr">
+        <is>
+          <t>COMISION MANTENIMIENTO</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1351,7 @@
         <f>F34+D35-E35</f>
         <v/>
       </c>
-      <c r="G35" s="20" t="inlineStr">
+      <c r="G35" s="21" t="inlineStr">
         <is>
           <t>Deposito en transito</t>
         </is>
@@ -1343,7 +1360,7 @@
     <row r="37">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>Saldo final según Mayor</t>
+          <t>Saldo Ajustado</t>
         </is>
       </c>
       <c r="F37" s="16">
@@ -1354,7 +1371,7 @@
     <row r="38">
       <c r="A38" s="17" t="inlineStr">
         <is>
-          <t>Saldo final según Banco</t>
+          <t>Saldo según Extracto</t>
         </is>
       </c>
       <c r="F38" s="16" t="n">
@@ -1368,7 +1385,7 @@
         </is>
       </c>
       <c r="F39" s="16">
-        <f>F38-F37</f>
+        <f>F37-F38</f>
         <v/>
       </c>
     </row>
@@ -1574,7 +1591,7 @@
         <v>46204</v>
       </c>
       <c r="B9" s="19" t="inlineStr"/>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>SALDO INICIAL</t>
         </is>
@@ -1589,19 +1606,19 @@
         <f>E9-D9</f>
         <v/>
       </c>
-      <c r="G9" s="20" t="inlineStr"/>
+      <c r="G9" s="21" t="inlineStr"/>
       <c r="H9" s="19" t="inlineStr"/>
-      <c r="I9" s="20" t="inlineStr"/>
+      <c r="I9" s="21" t="inlineStr"/>
       <c r="J9" s="19" t="inlineStr"/>
       <c r="K9" s="19" t="inlineStr">
         <is>
           <t>SANTANDER</t>
         </is>
       </c>
-      <c r="L9" s="20" t="inlineStr"/>
+      <c r="L9" s="21" t="inlineStr"/>
       <c r="M9" s="19" t="inlineStr"/>
-      <c r="N9" s="20" t="inlineStr"/>
-      <c r="O9" s="20" t="inlineStr"/>
+      <c r="N9" s="21" t="inlineStr"/>
+      <c r="O9" s="21" t="inlineStr"/>
       <c r="P9" s="19" t="inlineStr"/>
       <c r="Q9" s="19" t="inlineStr"/>
     </row>
@@ -1610,38 +1627,38 @@
         <v>46205</v>
       </c>
       <c r="B10" s="19" t="inlineStr"/>
-      <c r="C10" s="20" t="inlineStr">
+      <c r="C10" s="21" t="inlineStr">
         <is>
           <t>TRANSFERENCIA RECIBIDA CLIENTE NORTE</t>
         </is>
       </c>
-      <c r="D10" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="16" t="n">
+      <c r="D10" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="20" t="n">
         <v>1250000</v>
       </c>
       <c r="F10" s="16">
         <f>F9+E10-D10</f>
         <v/>
       </c>
-      <c r="G10" s="20" t="inlineStr"/>
+      <c r="G10" s="21" t="inlineStr"/>
       <c r="H10" s="19" t="inlineStr"/>
-      <c r="I10" s="20" t="inlineStr"/>
+      <c r="I10" s="21" t="inlineStr"/>
       <c r="J10" s="19" t="inlineStr"/>
       <c r="K10" s="19" t="inlineStr">
         <is>
           <t>SANTANDER</t>
         </is>
       </c>
-      <c r="L10" s="20" t="inlineStr"/>
+      <c r="L10" s="21" t="inlineStr"/>
       <c r="M10" s="19" t="inlineStr"/>
-      <c r="N10" s="20" t="inlineStr">
+      <c r="N10" s="21" t="inlineStr">
         <is>
           <t>TRF-88231</t>
         </is>
       </c>
-      <c r="O10" s="20" t="inlineStr"/>
+      <c r="O10" s="21" t="inlineStr"/>
       <c r="P10" s="19" t="inlineStr"/>
       <c r="Q10" s="19" t="inlineStr"/>
     </row>
@@ -1650,38 +1667,38 @@
         <v>46207</v>
       </c>
       <c r="B11" s="19" t="inlineStr"/>
-      <c r="C11" s="20" t="inlineStr">
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>PAGO PROVEEDOR LOGISTICA SRL</t>
         </is>
       </c>
-      <c r="D11" s="16" t="n">
+      <c r="D11" s="20" t="n">
         <v>320000</v>
       </c>
-      <c r="E11" s="16" t="n">
+      <c r="E11" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="16">
         <f>F10+E11-D11</f>
         <v/>
       </c>
-      <c r="G11" s="20" t="inlineStr"/>
+      <c r="G11" s="21" t="inlineStr"/>
       <c r="H11" s="19" t="inlineStr"/>
-      <c r="I11" s="20" t="inlineStr"/>
+      <c r="I11" s="21" t="inlineStr"/>
       <c r="J11" s="19" t="inlineStr"/>
       <c r="K11" s="19" t="inlineStr">
         <is>
           <t>SANTANDER</t>
         </is>
       </c>
-      <c r="L11" s="20" t="inlineStr"/>
+      <c r="L11" s="21" t="inlineStr"/>
       <c r="M11" s="19" t="inlineStr"/>
-      <c r="N11" s="20" t="inlineStr">
+      <c r="N11" s="21" t="inlineStr">
         <is>
           <t>CH-0000451</t>
         </is>
       </c>
-      <c r="O11" s="20" t="inlineStr"/>
+      <c r="O11" s="21" t="inlineStr"/>
       <c r="P11" s="19" t="inlineStr"/>
       <c r="Q11" s="19" t="inlineStr"/>
     </row>
@@ -1690,38 +1707,38 @@
         <v>46210</v>
       </c>
       <c r="B12" s="19" t="inlineStr"/>
-      <c r="C12" s="20" t="inlineStr">
+      <c r="C12" s="21" t="inlineStr">
         <is>
           <t>DEBITO AUTOMATICO EDESUR</t>
         </is>
       </c>
-      <c r="D12" s="16" t="n">
+      <c r="D12" s="20" t="n">
         <v>48200</v>
       </c>
-      <c r="E12" s="16" t="n">
+      <c r="E12" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="16">
         <f>F11+E12-D12</f>
         <v/>
       </c>
-      <c r="G12" s="20" t="inlineStr"/>
+      <c r="G12" s="21" t="inlineStr"/>
       <c r="H12" s="19" t="inlineStr"/>
-      <c r="I12" s="20" t="inlineStr"/>
+      <c r="I12" s="21" t="inlineStr"/>
       <c r="J12" s="19" t="inlineStr"/>
       <c r="K12" s="19" t="inlineStr">
         <is>
           <t>SANTANDER</t>
         </is>
       </c>
-      <c r="L12" s="20" t="inlineStr"/>
+      <c r="L12" s="21" t="inlineStr"/>
       <c r="M12" s="19" t="inlineStr"/>
-      <c r="N12" s="20" t="inlineStr">
+      <c r="N12" s="21" t="inlineStr">
         <is>
           <t>DB-77231</t>
         </is>
       </c>
-      <c r="O12" s="20" t="inlineStr"/>
+      <c r="O12" s="21" t="inlineStr"/>
       <c r="P12" s="19" t="inlineStr"/>
       <c r="Q12" s="19" t="inlineStr"/>
     </row>
@@ -1730,38 +1747,38 @@
         <v>46213</v>
       </c>
       <c r="B13" s="19" t="inlineStr"/>
-      <c r="C13" s="20" t="inlineStr">
+      <c r="C13" s="21" t="inlineStr">
         <is>
           <t>TRANSFERENCIA RECIBIDA CLIENTE CENTRO</t>
         </is>
       </c>
-      <c r="D13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="16" t="n">
+      <c r="D13" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="20" t="n">
         <v>530000</v>
       </c>
       <c r="F13" s="16">
         <f>F12+E13-D13</f>
         <v/>
       </c>
-      <c r="G13" s="20" t="inlineStr"/>
+      <c r="G13" s="21" t="inlineStr"/>
       <c r="H13" s="19" t="inlineStr"/>
-      <c r="I13" s="20" t="inlineStr"/>
+      <c r="I13" s="21" t="inlineStr"/>
       <c r="J13" s="19" t="inlineStr"/>
       <c r="K13" s="19" t="inlineStr">
         <is>
           <t>SANTANDER</t>
         </is>
       </c>
-      <c r="L13" s="20" t="inlineStr"/>
+      <c r="L13" s="21" t="inlineStr"/>
       <c r="M13" s="19" t="inlineStr"/>
-      <c r="N13" s="20" t="inlineStr">
+      <c r="N13" s="21" t="inlineStr">
         <is>
           <t>TRF-88245</t>
         </is>
       </c>
-      <c r="O13" s="20" t="inlineStr"/>
+      <c r="O13" s="21" t="inlineStr"/>
       <c r="P13" s="19" t="inlineStr"/>
       <c r="Q13" s="19" t="inlineStr"/>
     </row>
@@ -1770,38 +1787,38 @@
         <v>46215</v>
       </c>
       <c r="B14" s="19" t="inlineStr"/>
-      <c r="C14" s="20" t="inlineStr">
+      <c r="C14" s="21" t="inlineStr">
         <is>
           <t>TRANSFERENCIA SEGURO</t>
         </is>
       </c>
-      <c r="D14" s="16" t="n">
+      <c r="D14" s="20" t="n">
         <v>96000</v>
       </c>
-      <c r="E14" s="16" t="n">
+      <c r="E14" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="16">
         <f>F13+E14-D14</f>
         <v/>
       </c>
-      <c r="G14" s="20" t="inlineStr"/>
+      <c r="G14" s="21" t="inlineStr"/>
       <c r="H14" s="19" t="inlineStr"/>
-      <c r="I14" s="20" t="inlineStr"/>
+      <c r="I14" s="21" t="inlineStr"/>
       <c r="J14" s="19" t="inlineStr"/>
       <c r="K14" s="19" t="inlineStr">
         <is>
           <t>SANTANDER</t>
         </is>
       </c>
-      <c r="L14" s="20" t="inlineStr"/>
+      <c r="L14" s="21" t="inlineStr"/>
       <c r="M14" s="19" t="inlineStr"/>
-      <c r="N14" s="20" t="inlineStr">
+      <c r="N14" s="21" t="inlineStr">
         <is>
           <t>TRF-88251</t>
         </is>
       </c>
-      <c r="O14" s="20" t="inlineStr"/>
+      <c r="O14" s="21" t="inlineStr"/>
       <c r="P14" s="19" t="inlineStr"/>
       <c r="Q14" s="19" t="inlineStr"/>
     </row>
@@ -1810,38 +1827,38 @@
         <v>46218</v>
       </c>
       <c r="B15" s="19" t="inlineStr"/>
-      <c r="C15" s="20" t="inlineStr">
+      <c r="C15" s="21" t="inlineStr">
         <is>
           <t>TRANSFERENCIA RECIBIDA CLIENTE SUR</t>
         </is>
       </c>
-      <c r="D15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="16" t="n">
+      <c r="D15" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="20" t="n">
         <v>845000.5</v>
       </c>
       <c r="F15" s="16">
         <f>F14+E15-D15</f>
         <v/>
       </c>
-      <c r="G15" s="20" t="inlineStr"/>
+      <c r="G15" s="21" t="inlineStr"/>
       <c r="H15" s="19" t="inlineStr"/>
-      <c r="I15" s="20" t="inlineStr"/>
+      <c r="I15" s="21" t="inlineStr"/>
       <c r="J15" s="19" t="inlineStr"/>
       <c r="K15" s="19" t="inlineStr">
         <is>
           <t>SANTANDER</t>
         </is>
       </c>
-      <c r="L15" s="20" t="inlineStr"/>
+      <c r="L15" s="21" t="inlineStr"/>
       <c r="M15" s="19" t="inlineStr"/>
-      <c r="N15" s="20" t="inlineStr">
+      <c r="N15" s="21" t="inlineStr">
         <is>
           <t>TRF-88260</t>
         </is>
       </c>
-      <c r="O15" s="20" t="inlineStr"/>
+      <c r="O15" s="21" t="inlineStr"/>
       <c r="P15" s="19" t="inlineStr"/>
       <c r="Q15" s="19" t="inlineStr"/>
     </row>
@@ -1850,38 +1867,38 @@
         <v>46221</v>
       </c>
       <c r="B16" s="19" t="inlineStr"/>
-      <c r="C16" s="20" t="inlineStr">
+      <c r="C16" s="21" t="inlineStr">
         <is>
           <t>DEPOSITO EFECTIVO</t>
         </is>
       </c>
-      <c r="D16" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="16" t="n">
+      <c r="D16" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="20" t="n">
         <v>410000</v>
       </c>
       <c r="F16" s="16">
         <f>F15+E16-D16</f>
         <v/>
       </c>
-      <c r="G16" s="20" t="inlineStr"/>
+      <c r="G16" s="21" t="inlineStr"/>
       <c r="H16" s="19" t="inlineStr"/>
-      <c r="I16" s="20" t="inlineStr"/>
+      <c r="I16" s="21" t="inlineStr"/>
       <c r="J16" s="19" t="inlineStr"/>
       <c r="K16" s="19" t="inlineStr">
         <is>
           <t>SANTANDER</t>
         </is>
       </c>
-      <c r="L16" s="20" t="inlineStr"/>
+      <c r="L16" s="21" t="inlineStr"/>
       <c r="M16" s="19" t="inlineStr"/>
-      <c r="N16" s="20" t="inlineStr">
+      <c r="N16" s="21" t="inlineStr">
         <is>
           <t>DEP-0031</t>
         </is>
       </c>
-      <c r="O16" s="20" t="inlineStr"/>
+      <c r="O16" s="21" t="inlineStr"/>
       <c r="P16" s="19" t="inlineStr"/>
       <c r="Q16" s="19" t="inlineStr"/>
     </row>
@@ -1890,38 +1907,38 @@
         <v>46223</v>
       </c>
       <c r="B17" s="19" t="inlineStr"/>
-      <c r="C17" s="20" t="inlineStr">
+      <c r="C17" s="21" t="inlineStr">
         <is>
           <t>TRANSFERENCIA ALQUILER OFICINA</t>
         </is>
       </c>
-      <c r="D17" s="16" t="n">
+      <c r="D17" s="20" t="n">
         <v>250000</v>
       </c>
-      <c r="E17" s="16" t="n">
+      <c r="E17" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="16">
         <f>F16+E17-D17</f>
         <v/>
       </c>
-      <c r="G17" s="20" t="inlineStr"/>
+      <c r="G17" s="21" t="inlineStr"/>
       <c r="H17" s="19" t="inlineStr"/>
-      <c r="I17" s="20" t="inlineStr"/>
+      <c r="I17" s="21" t="inlineStr"/>
       <c r="J17" s="19" t="inlineStr"/>
       <c r="K17" s="19" t="inlineStr">
         <is>
           <t>SANTANDER</t>
         </is>
       </c>
-      <c r="L17" s="20" t="inlineStr"/>
+      <c r="L17" s="21" t="inlineStr"/>
       <c r="M17" s="19" t="inlineStr"/>
-      <c r="N17" s="20" t="inlineStr">
+      <c r="N17" s="21" t="inlineStr">
         <is>
           <t>TRF-88271</t>
         </is>
       </c>
-      <c r="O17" s="20" t="inlineStr"/>
+      <c r="O17" s="21" t="inlineStr"/>
       <c r="P17" s="19" t="inlineStr"/>
       <c r="Q17" s="19" t="inlineStr"/>
     </row>
@@ -1930,38 +1947,38 @@
         <v>46225</v>
       </c>
       <c r="B18" s="19" t="inlineStr"/>
-      <c r="C18" s="20" t="inlineStr">
+      <c r="C18" s="21" t="inlineStr">
         <is>
           <t>ACREDITACION INTERESES</t>
         </is>
       </c>
-      <c r="D18" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="16" t="n">
+      <c r="D18" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="20" t="n">
         <v>3200.25</v>
       </c>
       <c r="F18" s="16">
         <f>F17+E18-D18</f>
         <v/>
       </c>
-      <c r="G18" s="20" t="inlineStr"/>
+      <c r="G18" s="21" t="inlineStr"/>
       <c r="H18" s="19" t="inlineStr"/>
-      <c r="I18" s="20" t="inlineStr"/>
+      <c r="I18" s="21" t="inlineStr"/>
       <c r="J18" s="19" t="inlineStr"/>
       <c r="K18" s="19" t="inlineStr">
         <is>
           <t>SANTANDER</t>
         </is>
       </c>
-      <c r="L18" s="20" t="inlineStr"/>
+      <c r="L18" s="21" t="inlineStr"/>
       <c r="M18" s="19" t="inlineStr"/>
-      <c r="N18" s="20" t="inlineStr">
+      <c r="N18" s="21" t="inlineStr">
         <is>
           <t>INT-0004</t>
         </is>
       </c>
-      <c r="O18" s="20" t="inlineStr"/>
+      <c r="O18" s="21" t="inlineStr"/>
       <c r="P18" s="19" t="inlineStr"/>
       <c r="Q18" s="19" t="inlineStr"/>
     </row>
@@ -1970,38 +1987,38 @@
         <v>46228</v>
       </c>
       <c r="B19" s="19" t="inlineStr"/>
-      <c r="C19" s="20" t="inlineStr">
+      <c r="C19" s="21" t="inlineStr">
         <is>
           <t>TRANSFERENCIA RECIBIDA CLIENTE SUR</t>
         </is>
       </c>
-      <c r="D19" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="16" t="n">
+      <c r="D19" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="20" t="n">
         <v>275000</v>
       </c>
       <c r="F19" s="16">
         <f>F18+E19-D19</f>
         <v/>
       </c>
-      <c r="G19" s="20" t="inlineStr"/>
+      <c r="G19" s="21" t="inlineStr"/>
       <c r="H19" s="19" t="inlineStr"/>
-      <c r="I19" s="20" t="inlineStr"/>
+      <c r="I19" s="21" t="inlineStr"/>
       <c r="J19" s="19" t="inlineStr"/>
       <c r="K19" s="19" t="inlineStr">
         <is>
           <t>SANTANDER</t>
         </is>
       </c>
-      <c r="L19" s="20" t="inlineStr"/>
+      <c r="L19" s="21" t="inlineStr"/>
       <c r="M19" s="19" t="inlineStr"/>
-      <c r="N19" s="20" t="inlineStr">
+      <c r="N19" s="21" t="inlineStr">
         <is>
           <t>TRF-88290</t>
         </is>
       </c>
-      <c r="O19" s="20" t="inlineStr"/>
+      <c r="O19" s="21" t="inlineStr"/>
       <c r="P19" s="19" t="inlineStr"/>
       <c r="Q19" s="19" t="inlineStr"/>
     </row>
@@ -2010,38 +2027,38 @@
         <v>46231</v>
       </c>
       <c r="B20" s="19" t="inlineStr"/>
-      <c r="C20" s="20" t="inlineStr">
+      <c r="C20" s="21" t="inlineStr">
         <is>
           <t>PAGO PROVEEDOR INSUMOS SA</t>
         </is>
       </c>
-      <c r="D20" s="16" t="n">
+      <c r="D20" s="20" t="n">
         <v>198000</v>
       </c>
-      <c r="E20" s="16" t="n">
+      <c r="E20" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="16">
         <f>F19+E20-D20</f>
         <v/>
       </c>
-      <c r="G20" s="20" t="inlineStr"/>
+      <c r="G20" s="21" t="inlineStr"/>
       <c r="H20" s="19" t="inlineStr"/>
-      <c r="I20" s="20" t="inlineStr"/>
+      <c r="I20" s="21" t="inlineStr"/>
       <c r="J20" s="19" t="inlineStr"/>
       <c r="K20" s="19" t="inlineStr">
         <is>
           <t>SANTANDER</t>
         </is>
       </c>
-      <c r="L20" s="20" t="inlineStr"/>
+      <c r="L20" s="21" t="inlineStr"/>
       <c r="M20" s="19" t="inlineStr"/>
-      <c r="N20" s="20" t="inlineStr">
+      <c r="N20" s="21" t="inlineStr">
         <is>
           <t>CH-0000452</t>
         </is>
       </c>
-      <c r="O20" s="20" t="inlineStr"/>
+      <c r="O20" s="21" t="inlineStr"/>
       <c r="P20" s="19" t="inlineStr"/>
       <c r="Q20" s="19" t="inlineStr"/>
     </row>
@@ -2050,38 +2067,38 @@
         <v>46233</v>
       </c>
       <c r="B21" s="19" t="inlineStr"/>
-      <c r="C21" s="20" t="inlineStr">
+      <c r="C21" s="21" t="inlineStr">
         <is>
           <t>TRANSFERENCIA RECIBIDA CLIENTE CENTRO</t>
         </is>
       </c>
-      <c r="D21" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="16" t="n">
+      <c r="D21" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="20" t="n">
         <v>530000</v>
       </c>
       <c r="F21" s="16">
         <f>F20+E21-D21</f>
         <v/>
       </c>
-      <c r="G21" s="20" t="inlineStr"/>
+      <c r="G21" s="21" t="inlineStr"/>
       <c r="H21" s="19" t="inlineStr"/>
-      <c r="I21" s="20" t="inlineStr"/>
+      <c r="I21" s="21" t="inlineStr"/>
       <c r="J21" s="19" t="inlineStr"/>
       <c r="K21" s="19" t="inlineStr">
         <is>
           <t>SANTANDER</t>
         </is>
       </c>
-      <c r="L21" s="20" t="inlineStr"/>
+      <c r="L21" s="21" t="inlineStr"/>
       <c r="M21" s="19" t="inlineStr"/>
-      <c r="N21" s="20" t="inlineStr">
+      <c r="N21" s="21" t="inlineStr">
         <is>
           <t>TRF-88301</t>
         </is>
       </c>
-      <c r="O21" s="20" t="inlineStr"/>
+      <c r="O21" s="21" t="inlineStr"/>
       <c r="P21" s="19" t="inlineStr"/>
       <c r="Q21" s="19" t="inlineStr"/>
     </row>
@@ -2090,38 +2107,38 @@
         <v>46234</v>
       </c>
       <c r="B22" s="19" t="inlineStr"/>
-      <c r="C22" s="20" t="inlineStr">
+      <c r="C22" s="21" t="inlineStr">
         <is>
           <t>IMPUESTO LEY 25413</t>
         </is>
       </c>
-      <c r="D22" s="16" t="n">
+      <c r="D22" s="22" t="n">
         <v>9250</v>
       </c>
-      <c r="E22" s="16" t="n">
+      <c r="E22" s="22" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="16">
         <f>F21+E22-D22</f>
         <v/>
       </c>
-      <c r="G22" s="20" t="inlineStr"/>
+      <c r="G22" s="21" t="inlineStr"/>
       <c r="H22" s="19" t="inlineStr"/>
-      <c r="I22" s="20" t="inlineStr"/>
+      <c r="I22" s="21" t="inlineStr"/>
       <c r="J22" s="19" t="inlineStr"/>
       <c r="K22" s="19" t="inlineStr">
         <is>
           <t>SANTANDER</t>
         </is>
       </c>
-      <c r="L22" s="20" t="inlineStr"/>
+      <c r="L22" s="21" t="inlineStr"/>
       <c r="M22" s="19" t="inlineStr"/>
-      <c r="N22" s="20" t="inlineStr">
+      <c r="N22" s="21" t="inlineStr">
         <is>
           <t>IMP-0001</t>
         </is>
       </c>
-      <c r="O22" s="20" t="inlineStr"/>
+      <c r="O22" s="21" t="inlineStr"/>
       <c r="P22" s="19" t="inlineStr"/>
       <c r="Q22" s="19" t="inlineStr"/>
     </row>
@@ -2130,38 +2147,38 @@
         <v>46234</v>
       </c>
       <c r="B23" s="19" t="inlineStr"/>
-      <c r="C23" s="20" t="inlineStr">
+      <c r="C23" s="21" t="inlineStr">
         <is>
           <t>COMISION MANTENIMIENTO</t>
         </is>
       </c>
-      <c r="D23" s="16" t="n">
+      <c r="D23" s="22" t="n">
         <v>4800</v>
       </c>
-      <c r="E23" s="16" t="n">
+      <c r="E23" s="22" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="16">
         <f>F22+E23-D23</f>
         <v/>
       </c>
-      <c r="G23" s="20" t="inlineStr"/>
+      <c r="G23" s="21" t="inlineStr"/>
       <c r="H23" s="19" t="inlineStr"/>
-      <c r="I23" s="20" t="inlineStr"/>
+      <c r="I23" s="21" t="inlineStr"/>
       <c r="J23" s="19" t="inlineStr"/>
       <c r="K23" s="19" t="inlineStr">
         <is>
           <t>SANTANDER</t>
         </is>
       </c>
-      <c r="L23" s="20" t="inlineStr"/>
+      <c r="L23" s="21" t="inlineStr"/>
       <c r="M23" s="19" t="inlineStr"/>
-      <c r="N23" s="20" t="inlineStr">
+      <c r="N23" s="21" t="inlineStr">
         <is>
           <t>COM-0002</t>
         </is>
       </c>
-      <c r="O23" s="20" t="inlineStr"/>
+      <c r="O23" s="21" t="inlineStr"/>
       <c r="P23" s="19" t="inlineStr"/>
       <c r="Q23" s="19" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Export FO 02-03: verde claro y resaltado de una sola celda
El rosado de los debitos del banco pendientes pasa al verde claro del formulario real (#93C47D) y el resaltado cubre solo la celda del importe que tiene valor (Debe o Haber), no las dos columnas.
</commit_message>
<xml_diff>
--- a/FO_02-03_DEMO.xlsx
+++ b/FO_02-03_DEMO.xlsx
@@ -60,7 +60,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD5A6BD"/>
+        <fgColor rgb="FF93C47D"/>
       </patternFill>
     </fill>
   </fills>
@@ -725,7 +725,7 @@
       <c r="D10" s="20" t="n">
         <v>1250000</v>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E10" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="16">
@@ -750,7 +750,7 @@
         </is>
       </c>
       <c r="C11" s="19" t="inlineStr"/>
-      <c r="D11" s="20" t="n">
+      <c r="D11" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="20" t="n">
@@ -781,7 +781,7 @@
       <c r="D12" s="20" t="n">
         <v>845000.5</v>
       </c>
-      <c r="E12" s="20" t="n">
+      <c r="E12" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="16">
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr"/>
-      <c r="D13" s="20" t="n">
+      <c r="D13" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="20" t="n">
@@ -834,7 +834,7 @@
         </is>
       </c>
       <c r="C14" s="19" t="inlineStr"/>
-      <c r="D14" s="20" t="n">
+      <c r="D14" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="20" t="n">
@@ -865,7 +865,7 @@
       <c r="D15" s="20" t="n">
         <v>15500.75</v>
       </c>
-      <c r="E15" s="20" t="n">
+      <c r="E15" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="16">
@@ -893,7 +893,7 @@
       <c r="D16" s="20" t="n">
         <v>530000</v>
       </c>
-      <c r="E16" s="20" t="n">
+      <c r="E16" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="16">
@@ -918,7 +918,7 @@
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr"/>
-      <c r="D17" s="20" t="n">
+      <c r="D17" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E17" s="20" t="n">
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="C18" s="19" t="inlineStr"/>
-      <c r="D18" s="20" t="n">
+      <c r="D18" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="20" t="n">
@@ -977,7 +977,7 @@
       <c r="D19" s="20" t="n">
         <v>410000</v>
       </c>
-      <c r="E19" s="20" t="n">
+      <c r="E19" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="16">
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="C20" s="19" t="inlineStr"/>
-      <c r="D20" s="20" t="n">
+      <c r="D20" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="20" t="n">
@@ -1030,7 +1030,7 @@
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr"/>
-      <c r="D21" s="20" t="n">
+      <c r="D21" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="20" t="n">
@@ -1061,7 +1061,7 @@
       <c r="D22" s="20" t="n">
         <v>275000</v>
       </c>
-      <c r="E22" s="20" t="n">
+      <c r="E22" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="16">
@@ -1086,7 +1086,7 @@
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr"/>
-      <c r="D23" s="20" t="n">
+      <c r="D23" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E23" s="20" t="n">
@@ -1632,7 +1632,7 @@
           <t>TRANSFERENCIA RECIBIDA CLIENTE NORTE</t>
         </is>
       </c>
-      <c r="D10" s="20" t="n">
+      <c r="D10" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="20" t="n">
@@ -1675,7 +1675,7 @@
       <c r="D11" s="20" t="n">
         <v>320000</v>
       </c>
-      <c r="E11" s="20" t="n">
+      <c r="E11" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="16">
@@ -1715,7 +1715,7 @@
       <c r="D12" s="20" t="n">
         <v>48200</v>
       </c>
-      <c r="E12" s="20" t="n">
+      <c r="E12" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="16">
@@ -1752,7 +1752,7 @@
           <t>TRANSFERENCIA RECIBIDA CLIENTE CENTRO</t>
         </is>
       </c>
-      <c r="D13" s="20" t="n">
+      <c r="D13" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="20" t="n">
@@ -1795,7 +1795,7 @@
       <c r="D14" s="20" t="n">
         <v>96000</v>
       </c>
-      <c r="E14" s="20" t="n">
+      <c r="E14" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="16">
@@ -1832,7 +1832,7 @@
           <t>TRANSFERENCIA RECIBIDA CLIENTE SUR</t>
         </is>
       </c>
-      <c r="D15" s="20" t="n">
+      <c r="D15" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="20" t="n">
@@ -1872,7 +1872,7 @@
           <t>DEPOSITO EFECTIVO</t>
         </is>
       </c>
-      <c r="D16" s="20" t="n">
+      <c r="D16" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E16" s="20" t="n">
@@ -1915,7 +1915,7 @@
       <c r="D17" s="20" t="n">
         <v>250000</v>
       </c>
-      <c r="E17" s="20" t="n">
+      <c r="E17" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="16">
@@ -1952,7 +1952,7 @@
           <t>ACREDITACION INTERESES</t>
         </is>
       </c>
-      <c r="D18" s="20" t="n">
+      <c r="D18" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="20" t="n">
@@ -1992,7 +1992,7 @@
           <t>TRANSFERENCIA RECIBIDA CLIENTE SUR</t>
         </is>
       </c>
-      <c r="D19" s="20" t="n">
+      <c r="D19" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E19" s="20" t="n">
@@ -2035,7 +2035,7 @@
       <c r="D20" s="20" t="n">
         <v>198000</v>
       </c>
-      <c r="E20" s="20" t="n">
+      <c r="E20" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="16">
@@ -2072,7 +2072,7 @@
           <t>TRANSFERENCIA RECIBIDA CLIENTE CENTRO</t>
         </is>
       </c>
-      <c r="D21" s="20" t="n">
+      <c r="D21" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="20" t="n">
@@ -2115,7 +2115,7 @@
       <c r="D22" s="22" t="n">
         <v>9250</v>
       </c>
-      <c r="E22" s="22" t="n">
+      <c r="E22" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="16">
@@ -2155,7 +2155,7 @@
       <c r="D23" s="22" t="n">
         <v>4800</v>
       </c>
-      <c r="E23" s="22" t="n">
+      <c r="E23" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="16">

</xml_diff>

<commit_message>
Export FO 02-03: Seccion 3 con gastos bancarios, Haber, total y verde en el origen
</commit_message>
<xml_diff>
--- a/FO_02-03_DEMO.xlsx
+++ b/FO_02-03_DEMO.xlsx
@@ -1289,14 +1289,12 @@
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr"/>
-      <c r="D33" s="16" t="n">
+      <c r="D33" s="21" t="n"/>
+      <c r="E33" s="16" t="n">
         <v>9250</v>
       </c>
-      <c r="E33" s="16" t="n">
-        <v>0</v>
-      </c>
       <c r="F33" s="16">
-        <f>D33-E33</f>
+        <f>F32+D33-E33</f>
         <v/>
       </c>
       <c r="G33" s="21" t="inlineStr">
@@ -1315,11 +1313,9 @@
         </is>
       </c>
       <c r="C34" s="19" t="inlineStr"/>
-      <c r="D34" s="16" t="n">
+      <c r="D34" s="21" t="n"/>
+      <c r="E34" s="16" t="n">
         <v>4800</v>
-      </c>
-      <c r="E34" s="16" t="n">
-        <v>0</v>
       </c>
       <c r="F34" s="16">
         <f>F33+D34-E34</f>
@@ -1332,29 +1328,14 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="18" t="n">
-        <v>46234</v>
-      </c>
-      <c r="B35" s="19" t="inlineStr">
-        <is>
-          <t>DEP-0003</t>
-        </is>
-      </c>
-      <c r="C35" s="19" t="inlineStr"/>
-      <c r="D35" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" s="16" t="n">
-        <v>300000</v>
-      </c>
-      <c r="F35" s="16">
-        <f>F34+D35-E35</f>
-        <v/>
-      </c>
-      <c r="G35" s="21" t="inlineStr">
-        <is>
-          <t>Deposito en transito</t>
-        </is>
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>Total gastos e impuestos pendientes</t>
+        </is>
+      </c>
+      <c r="E35" s="16">
+        <f>SUM(E33:E34)</f>
+        <v/>
       </c>
     </row>
     <row r="37">

</xml_diff>

<commit_message>
Export FO 02-03: fila TOTALES en Movimientos, sin control y dedupe del extracto
</commit_message>
<xml_diff>
--- a/FO_02-03_DEMO.xlsx
+++ b/FO_02-03_DEMO.xlsx
@@ -2166,11 +2166,19 @@
     <row r="24">
       <c r="A24" s="17" t="inlineStr">
         <is>
-          <t>Control de diferencia</t>
-        </is>
+          <t>TOTALES</t>
+        </is>
+      </c>
+      <c r="D24" s="16">
+        <f>SUM(D9:D23)</f>
+        <v/>
+      </c>
+      <c r="E24" s="16">
+        <f>SUM(E9:E23)</f>
+        <v/>
       </c>
       <c r="F24" s="16">
-        <f>F23-'Libro Mayor'!F24</f>
+        <f>F23</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Export FO 02-03: Movimientos Bancarios en 5 columnas (fecha, concepto, debito, credito, saldo)
</commit_message>
<xml_diff>
--- a/FO_02-03_DEMO.xlsx
+++ b/FO_02-03_DEMO.xlsx
@@ -1385,26 +1385,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="24" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -1488,82 +1476,22 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Cod de Concepto</t>
+          <t>Concepto</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Concepto</t>
+          <t>Debito en $</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>Debito en $</t>
+          <t>Credito en $</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>Credito en $</t>
-        </is>
-      </c>
-      <c r="F8" s="15" t="inlineStr">
-        <is>
           <t>Saldo en $</t>
-        </is>
-      </c>
-      <c r="G8" s="15" t="inlineStr">
-        <is>
-          <t>Informacion Complementaria</t>
-        </is>
-      </c>
-      <c r="H8" s="15" t="inlineStr">
-        <is>
-          <t>Nro de cheque</t>
-        </is>
-      </c>
-      <c r="I8" s="15" t="inlineStr">
-        <is>
-          <t>Sucursal Origen</t>
-        </is>
-      </c>
-      <c r="J8" s="15" t="inlineStr">
-        <is>
-          <t>Canal</t>
-        </is>
-      </c>
-      <c r="K8" s="15" t="inlineStr">
-        <is>
-          <t>Banco</t>
-        </is>
-      </c>
-      <c r="L8" s="15" t="inlineStr">
-        <is>
-          <t>CBU/Alias</t>
-        </is>
-      </c>
-      <c r="M8" s="15" t="inlineStr">
-        <is>
-          <t>Tipo trf</t>
-        </is>
-      </c>
-      <c r="N8" s="15" t="inlineStr">
-        <is>
-          <t>Referencia</t>
-        </is>
-      </c>
-      <c r="O8" s="15" t="inlineStr">
-        <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="P8" s="15" t="inlineStr">
-        <is>
-          <t>Tipo doc</t>
-        </is>
-      </c>
-      <c r="Q8" s="15" t="inlineStr">
-        <is>
-          <t>Nro doc</t>
         </is>
       </c>
     </row>
@@ -1571,597 +1499,301 @@
       <c r="A9" s="18" t="n">
         <v>46204</v>
       </c>
-      <c r="B9" s="19" t="inlineStr"/>
-      <c r="C9" s="21" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>SALDO INICIAL</t>
         </is>
       </c>
+      <c r="C9" s="16" t="n">
+        <v>0</v>
+      </c>
       <c r="D9" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="16">
-        <f>E9-D9</f>
-        <v/>
-      </c>
-      <c r="G9" s="21" t="inlineStr"/>
-      <c r="H9" s="19" t="inlineStr"/>
-      <c r="I9" s="21" t="inlineStr"/>
-      <c r="J9" s="19" t="inlineStr"/>
-      <c r="K9" s="19" t="inlineStr">
-        <is>
-          <t>SANTANDER</t>
-        </is>
-      </c>
-      <c r="L9" s="21" t="inlineStr"/>
-      <c r="M9" s="19" t="inlineStr"/>
-      <c r="N9" s="21" t="inlineStr"/>
-      <c r="O9" s="21" t="inlineStr"/>
-      <c r="P9" s="19" t="inlineStr"/>
-      <c r="Q9" s="19" t="inlineStr"/>
+      <c r="E9" s="16">
+        <f>D9-C9</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="18" t="n">
         <v>46205</v>
       </c>
-      <c r="B10" s="19" t="inlineStr"/>
-      <c r="C10" s="21" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>TRANSFERENCIA RECIBIDA CLIENTE NORTE</t>
         </is>
       </c>
-      <c r="D10" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="20" t="n">
+      <c r="C10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="20" t="n">
         <v>1250000</v>
       </c>
-      <c r="F10" s="16">
-        <f>F9+E10-D10</f>
-        <v/>
-      </c>
-      <c r="G10" s="21" t="inlineStr"/>
-      <c r="H10" s="19" t="inlineStr"/>
-      <c r="I10" s="21" t="inlineStr"/>
-      <c r="J10" s="19" t="inlineStr"/>
-      <c r="K10" s="19" t="inlineStr">
-        <is>
-          <t>SANTANDER</t>
-        </is>
-      </c>
-      <c r="L10" s="21" t="inlineStr"/>
-      <c r="M10" s="19" t="inlineStr"/>
-      <c r="N10" s="21" t="inlineStr">
-        <is>
-          <t>TRF-88231</t>
-        </is>
-      </c>
-      <c r="O10" s="21" t="inlineStr"/>
-      <c r="P10" s="19" t="inlineStr"/>
-      <c r="Q10" s="19" t="inlineStr"/>
+      <c r="E10" s="16">
+        <f>E9+D10-C10</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="18" t="n">
         <v>46207</v>
       </c>
-      <c r="B11" s="19" t="inlineStr"/>
-      <c r="C11" s="21" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>PAGO PROVEEDOR LOGISTICA SRL</t>
         </is>
       </c>
-      <c r="D11" s="20" t="n">
+      <c r="C11" s="20" t="n">
         <v>320000</v>
       </c>
-      <c r="E11" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="16">
-        <f>F10+E11-D11</f>
-        <v/>
-      </c>
-      <c r="G11" s="21" t="inlineStr"/>
-      <c r="H11" s="19" t="inlineStr"/>
-      <c r="I11" s="21" t="inlineStr"/>
-      <c r="J11" s="19" t="inlineStr"/>
-      <c r="K11" s="19" t="inlineStr">
-        <is>
-          <t>SANTANDER</t>
-        </is>
-      </c>
-      <c r="L11" s="21" t="inlineStr"/>
-      <c r="M11" s="19" t="inlineStr"/>
-      <c r="N11" s="21" t="inlineStr">
-        <is>
-          <t>CH-0000451</t>
-        </is>
-      </c>
-      <c r="O11" s="21" t="inlineStr"/>
-      <c r="P11" s="19" t="inlineStr"/>
-      <c r="Q11" s="19" t="inlineStr"/>
+      <c r="D11" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="16">
+        <f>E10+D11-C11</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="18" t="n">
         <v>46210</v>
       </c>
-      <c r="B12" s="19" t="inlineStr"/>
-      <c r="C12" s="21" t="inlineStr">
+      <c r="B12" s="19" t="inlineStr">
         <is>
           <t>DEBITO AUTOMATICO EDESUR</t>
         </is>
       </c>
-      <c r="D12" s="20" t="n">
+      <c r="C12" s="20" t="n">
         <v>48200</v>
       </c>
-      <c r="E12" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="16">
-        <f>F11+E12-D12</f>
-        <v/>
-      </c>
-      <c r="G12" s="21" t="inlineStr"/>
-      <c r="H12" s="19" t="inlineStr"/>
-      <c r="I12" s="21" t="inlineStr"/>
-      <c r="J12" s="19" t="inlineStr"/>
-      <c r="K12" s="19" t="inlineStr">
-        <is>
-          <t>SANTANDER</t>
-        </is>
-      </c>
-      <c r="L12" s="21" t="inlineStr"/>
-      <c r="M12" s="19" t="inlineStr"/>
-      <c r="N12" s="21" t="inlineStr">
-        <is>
-          <t>DB-77231</t>
-        </is>
-      </c>
-      <c r="O12" s="21" t="inlineStr"/>
-      <c r="P12" s="19" t="inlineStr"/>
-      <c r="Q12" s="19" t="inlineStr"/>
+      <c r="D12" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="16">
+        <f>E11+D12-C12</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="18" t="n">
         <v>46213</v>
       </c>
-      <c r="B13" s="19" t="inlineStr"/>
-      <c r="C13" s="21" t="inlineStr">
+      <c r="B13" s="19" t="inlineStr">
         <is>
           <t>TRANSFERENCIA RECIBIDA CLIENTE CENTRO</t>
         </is>
       </c>
-      <c r="D13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="20" t="n">
+      <c r="C13" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="20" t="n">
         <v>530000</v>
       </c>
-      <c r="F13" s="16">
-        <f>F12+E13-D13</f>
-        <v/>
-      </c>
-      <c r="G13" s="21" t="inlineStr"/>
-      <c r="H13" s="19" t="inlineStr"/>
-      <c r="I13" s="21" t="inlineStr"/>
-      <c r="J13" s="19" t="inlineStr"/>
-      <c r="K13" s="19" t="inlineStr">
-        <is>
-          <t>SANTANDER</t>
-        </is>
-      </c>
-      <c r="L13" s="21" t="inlineStr"/>
-      <c r="M13" s="19" t="inlineStr"/>
-      <c r="N13" s="21" t="inlineStr">
-        <is>
-          <t>TRF-88245</t>
-        </is>
-      </c>
-      <c r="O13" s="21" t="inlineStr"/>
-      <c r="P13" s="19" t="inlineStr"/>
-      <c r="Q13" s="19" t="inlineStr"/>
+      <c r="E13" s="16">
+        <f>E12+D13-C13</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="18" t="n">
         <v>46215</v>
       </c>
-      <c r="B14" s="19" t="inlineStr"/>
-      <c r="C14" s="21" t="inlineStr">
+      <c r="B14" s="19" t="inlineStr">
         <is>
           <t>TRANSFERENCIA SEGURO</t>
         </is>
       </c>
-      <c r="D14" s="20" t="n">
+      <c r="C14" s="20" t="n">
         <v>96000</v>
       </c>
-      <c r="E14" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="16">
-        <f>F13+E14-D14</f>
-        <v/>
-      </c>
-      <c r="G14" s="21" t="inlineStr"/>
-      <c r="H14" s="19" t="inlineStr"/>
-      <c r="I14" s="21" t="inlineStr"/>
-      <c r="J14" s="19" t="inlineStr"/>
-      <c r="K14" s="19" t="inlineStr">
-        <is>
-          <t>SANTANDER</t>
-        </is>
-      </c>
-      <c r="L14" s="21" t="inlineStr"/>
-      <c r="M14" s="19" t="inlineStr"/>
-      <c r="N14" s="21" t="inlineStr">
-        <is>
-          <t>TRF-88251</t>
-        </is>
-      </c>
-      <c r="O14" s="21" t="inlineStr"/>
-      <c r="P14" s="19" t="inlineStr"/>
-      <c r="Q14" s="19" t="inlineStr"/>
+      <c r="D14" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="16">
+        <f>E13+D14-C14</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="18" t="n">
         <v>46218</v>
       </c>
-      <c r="B15" s="19" t="inlineStr"/>
-      <c r="C15" s="21" t="inlineStr">
+      <c r="B15" s="19" t="inlineStr">
         <is>
           <t>TRANSFERENCIA RECIBIDA CLIENTE SUR</t>
         </is>
       </c>
-      <c r="D15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="20" t="n">
+      <c r="C15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="20" t="n">
         <v>845000.5</v>
       </c>
-      <c r="F15" s="16">
-        <f>F14+E15-D15</f>
-        <v/>
-      </c>
-      <c r="G15" s="21" t="inlineStr"/>
-      <c r="H15" s="19" t="inlineStr"/>
-      <c r="I15" s="21" t="inlineStr"/>
-      <c r="J15" s="19" t="inlineStr"/>
-      <c r="K15" s="19" t="inlineStr">
-        <is>
-          <t>SANTANDER</t>
-        </is>
-      </c>
-      <c r="L15" s="21" t="inlineStr"/>
-      <c r="M15" s="19" t="inlineStr"/>
-      <c r="N15" s="21" t="inlineStr">
-        <is>
-          <t>TRF-88260</t>
-        </is>
-      </c>
-      <c r="O15" s="21" t="inlineStr"/>
-      <c r="P15" s="19" t="inlineStr"/>
-      <c r="Q15" s="19" t="inlineStr"/>
+      <c r="E15" s="16">
+        <f>E14+D15-C15</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="18" t="n">
         <v>46221</v>
       </c>
-      <c r="B16" s="19" t="inlineStr"/>
-      <c r="C16" s="21" t="inlineStr">
+      <c r="B16" s="19" t="inlineStr">
         <is>
           <t>DEPOSITO EFECTIVO</t>
         </is>
       </c>
-      <c r="D16" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="20" t="n">
+      <c r="C16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="20" t="n">
         <v>410000</v>
       </c>
-      <c r="F16" s="16">
-        <f>F15+E16-D16</f>
-        <v/>
-      </c>
-      <c r="G16" s="21" t="inlineStr"/>
-      <c r="H16" s="19" t="inlineStr"/>
-      <c r="I16" s="21" t="inlineStr"/>
-      <c r="J16" s="19" t="inlineStr"/>
-      <c r="K16" s="19" t="inlineStr">
-        <is>
-          <t>SANTANDER</t>
-        </is>
-      </c>
-      <c r="L16" s="21" t="inlineStr"/>
-      <c r="M16" s="19" t="inlineStr"/>
-      <c r="N16" s="21" t="inlineStr">
-        <is>
-          <t>DEP-0031</t>
-        </is>
-      </c>
-      <c r="O16" s="21" t="inlineStr"/>
-      <c r="P16" s="19" t="inlineStr"/>
-      <c r="Q16" s="19" t="inlineStr"/>
+      <c r="E16" s="16">
+        <f>E15+D16-C16</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="18" t="n">
         <v>46223</v>
       </c>
-      <c r="B17" s="19" t="inlineStr"/>
-      <c r="C17" s="21" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>TRANSFERENCIA ALQUILER OFICINA</t>
         </is>
       </c>
-      <c r="D17" s="20" t="n">
+      <c r="C17" s="20" t="n">
         <v>250000</v>
       </c>
-      <c r="E17" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="16">
-        <f>F16+E17-D17</f>
-        <v/>
-      </c>
-      <c r="G17" s="21" t="inlineStr"/>
-      <c r="H17" s="19" t="inlineStr"/>
-      <c r="I17" s="21" t="inlineStr"/>
-      <c r="J17" s="19" t="inlineStr"/>
-      <c r="K17" s="19" t="inlineStr">
-        <is>
-          <t>SANTANDER</t>
-        </is>
-      </c>
-      <c r="L17" s="21" t="inlineStr"/>
-      <c r="M17" s="19" t="inlineStr"/>
-      <c r="N17" s="21" t="inlineStr">
-        <is>
-          <t>TRF-88271</t>
-        </is>
-      </c>
-      <c r="O17" s="21" t="inlineStr"/>
-      <c r="P17" s="19" t="inlineStr"/>
-      <c r="Q17" s="19" t="inlineStr"/>
+      <c r="D17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="16">
+        <f>E16+D17-C17</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="18" t="n">
         <v>46225</v>
       </c>
-      <c r="B18" s="19" t="inlineStr"/>
-      <c r="C18" s="21" t="inlineStr">
+      <c r="B18" s="19" t="inlineStr">
         <is>
           <t>ACREDITACION INTERESES</t>
         </is>
       </c>
-      <c r="D18" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="20" t="n">
+      <c r="C18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="20" t="n">
         <v>3200.25</v>
       </c>
-      <c r="F18" s="16">
-        <f>F17+E18-D18</f>
-        <v/>
-      </c>
-      <c r="G18" s="21" t="inlineStr"/>
-      <c r="H18" s="19" t="inlineStr"/>
-      <c r="I18" s="21" t="inlineStr"/>
-      <c r="J18" s="19" t="inlineStr"/>
-      <c r="K18" s="19" t="inlineStr">
-        <is>
-          <t>SANTANDER</t>
-        </is>
-      </c>
-      <c r="L18" s="21" t="inlineStr"/>
-      <c r="M18" s="19" t="inlineStr"/>
-      <c r="N18" s="21" t="inlineStr">
-        <is>
-          <t>INT-0004</t>
-        </is>
-      </c>
-      <c r="O18" s="21" t="inlineStr"/>
-      <c r="P18" s="19" t="inlineStr"/>
-      <c r="Q18" s="19" t="inlineStr"/>
+      <c r="E18" s="16">
+        <f>E17+D18-C18</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="18" t="n">
         <v>46228</v>
       </c>
-      <c r="B19" s="19" t="inlineStr"/>
-      <c r="C19" s="21" t="inlineStr">
+      <c r="B19" s="19" t="inlineStr">
         <is>
           <t>TRANSFERENCIA RECIBIDA CLIENTE SUR</t>
         </is>
       </c>
-      <c r="D19" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="20" t="n">
+      <c r="C19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="20" t="n">
         <v>275000</v>
       </c>
-      <c r="F19" s="16">
-        <f>F18+E19-D19</f>
-        <v/>
-      </c>
-      <c r="G19" s="21" t="inlineStr"/>
-      <c r="H19" s="19" t="inlineStr"/>
-      <c r="I19" s="21" t="inlineStr"/>
-      <c r="J19" s="19" t="inlineStr"/>
-      <c r="K19" s="19" t="inlineStr">
-        <is>
-          <t>SANTANDER</t>
-        </is>
-      </c>
-      <c r="L19" s="21" t="inlineStr"/>
-      <c r="M19" s="19" t="inlineStr"/>
-      <c r="N19" s="21" t="inlineStr">
-        <is>
-          <t>TRF-88290</t>
-        </is>
-      </c>
-      <c r="O19" s="21" t="inlineStr"/>
-      <c r="P19" s="19" t="inlineStr"/>
-      <c r="Q19" s="19" t="inlineStr"/>
+      <c r="E19" s="16">
+        <f>E18+D19-C19</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="18" t="n">
         <v>46231</v>
       </c>
-      <c r="B20" s="19" t="inlineStr"/>
-      <c r="C20" s="21" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>PAGO PROVEEDOR INSUMOS SA</t>
         </is>
       </c>
-      <c r="D20" s="20" t="n">
+      <c r="C20" s="20" t="n">
         <v>198000</v>
       </c>
-      <c r="E20" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="16">
-        <f>F19+E20-D20</f>
-        <v/>
-      </c>
-      <c r="G20" s="21" t="inlineStr"/>
-      <c r="H20" s="19" t="inlineStr"/>
-      <c r="I20" s="21" t="inlineStr"/>
-      <c r="J20" s="19" t="inlineStr"/>
-      <c r="K20" s="19" t="inlineStr">
-        <is>
-          <t>SANTANDER</t>
-        </is>
-      </c>
-      <c r="L20" s="21" t="inlineStr"/>
-      <c r="M20" s="19" t="inlineStr"/>
-      <c r="N20" s="21" t="inlineStr">
-        <is>
-          <t>CH-0000452</t>
-        </is>
-      </c>
-      <c r="O20" s="21" t="inlineStr"/>
-      <c r="P20" s="19" t="inlineStr"/>
-      <c r="Q20" s="19" t="inlineStr"/>
+      <c r="D20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="16">
+        <f>E19+D20-C20</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="18" t="n">
         <v>46233</v>
       </c>
-      <c r="B21" s="19" t="inlineStr"/>
-      <c r="C21" s="21" t="inlineStr">
+      <c r="B21" s="19" t="inlineStr">
         <is>
           <t>TRANSFERENCIA RECIBIDA CLIENTE CENTRO</t>
         </is>
       </c>
-      <c r="D21" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="20" t="n">
+      <c r="C21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="20" t="n">
         <v>530000</v>
       </c>
-      <c r="F21" s="16">
-        <f>F20+E21-D21</f>
-        <v/>
-      </c>
-      <c r="G21" s="21" t="inlineStr"/>
-      <c r="H21" s="19" t="inlineStr"/>
-      <c r="I21" s="21" t="inlineStr"/>
-      <c r="J21" s="19" t="inlineStr"/>
-      <c r="K21" s="19" t="inlineStr">
-        <is>
-          <t>SANTANDER</t>
-        </is>
-      </c>
-      <c r="L21" s="21" t="inlineStr"/>
-      <c r="M21" s="19" t="inlineStr"/>
-      <c r="N21" s="21" t="inlineStr">
-        <is>
-          <t>TRF-88301</t>
-        </is>
-      </c>
-      <c r="O21" s="21" t="inlineStr"/>
-      <c r="P21" s="19" t="inlineStr"/>
-      <c r="Q21" s="19" t="inlineStr"/>
+      <c r="E21" s="16">
+        <f>E20+D21-C21</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="18" t="n">
         <v>46234</v>
       </c>
-      <c r="B22" s="19" t="inlineStr"/>
-      <c r="C22" s="21" t="inlineStr">
+      <c r="B22" s="19" t="inlineStr">
         <is>
           <t>IMPUESTO LEY 25413</t>
         </is>
       </c>
-      <c r="D22" s="22" t="n">
+      <c r="C22" s="22" t="n">
         <v>9250</v>
       </c>
-      <c r="E22" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="16">
-        <f>F21+E22-D22</f>
-        <v/>
-      </c>
-      <c r="G22" s="21" t="inlineStr"/>
-      <c r="H22" s="19" t="inlineStr"/>
-      <c r="I22" s="21" t="inlineStr"/>
-      <c r="J22" s="19" t="inlineStr"/>
-      <c r="K22" s="19" t="inlineStr">
-        <is>
-          <t>SANTANDER</t>
-        </is>
-      </c>
-      <c r="L22" s="21" t="inlineStr"/>
-      <c r="M22" s="19" t="inlineStr"/>
-      <c r="N22" s="21" t="inlineStr">
-        <is>
-          <t>IMP-0001</t>
-        </is>
-      </c>
-      <c r="O22" s="21" t="inlineStr"/>
-      <c r="P22" s="19" t="inlineStr"/>
-      <c r="Q22" s="19" t="inlineStr"/>
+      <c r="D22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="16">
+        <f>E21+D22-C22</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="18" t="n">
         <v>46234</v>
       </c>
-      <c r="B23" s="19" t="inlineStr"/>
-      <c r="C23" s="21" t="inlineStr">
+      <c r="B23" s="19" t="inlineStr">
         <is>
           <t>COMISION MANTENIMIENTO</t>
         </is>
       </c>
-      <c r="D23" s="22" t="n">
+      <c r="C23" s="22" t="n">
         <v>4800</v>
       </c>
-      <c r="E23" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="16">
-        <f>F22+E23-D23</f>
-        <v/>
-      </c>
-      <c r="G23" s="21" t="inlineStr"/>
-      <c r="H23" s="19" t="inlineStr"/>
-      <c r="I23" s="21" t="inlineStr"/>
-      <c r="J23" s="19" t="inlineStr"/>
-      <c r="K23" s="19" t="inlineStr">
-        <is>
-          <t>SANTANDER</t>
-        </is>
-      </c>
-      <c r="L23" s="21" t="inlineStr"/>
-      <c r="M23" s="19" t="inlineStr"/>
-      <c r="N23" s="21" t="inlineStr">
-        <is>
-          <t>COM-0002</t>
-        </is>
-      </c>
-      <c r="O23" s="21" t="inlineStr"/>
-      <c r="P23" s="19" t="inlineStr"/>
-      <c r="Q23" s="19" t="inlineStr"/>
+      <c r="D23" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="16">
+        <f>E22+D23-C23</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="17" t="inlineStr">
@@ -2169,16 +1801,16 @@
           <t>TOTALES</t>
         </is>
       </c>
+      <c r="C24" s="16">
+        <f>SUM(C9:C23)</f>
+        <v/>
+      </c>
       <c r="D24" s="16">
         <f>SUM(D9:D23)</f>
         <v/>
       </c>
       <c r="E24" s="16">
-        <f>SUM(E9:E23)</f>
-        <v/>
-      </c>
-      <c r="F24" s="16">
-        <f>F23</f>
+        <f>E23</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Export FO 02-03: cuadro de totales al lado en Movimientos, sin fila TOTALES
</commit_message>
<xml_diff>
--- a/FO_02-03_DEMO.xlsx
+++ b/FO_02-03_DEMO.xlsx
@@ -147,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -197,6 +197,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" shrinkToFit="1"/>
@@ -1385,7 +1391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1393,6 +1399,8 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -1494,6 +1502,15 @@
           <t>Saldo en $</t>
         </is>
       </c>
+      <c r="G8" s="22" t="inlineStr">
+        <is>
+          <t>Total Débitos</t>
+        </is>
+      </c>
+      <c r="H8" s="23">
+        <f>SUM(C9:C23)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="18" t="n">
@@ -1514,6 +1531,15 @@
         <f>D9-C9</f>
         <v/>
       </c>
+      <c r="G9" s="22" t="inlineStr">
+        <is>
+          <t>Total Créditos</t>
+        </is>
+      </c>
+      <c r="H9" s="23">
+        <f>SUM(D9:D23)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="18" t="n">
@@ -1764,7 +1790,7 @@
           <t>IMPUESTO LEY 25413</t>
         </is>
       </c>
-      <c r="C22" s="22" t="n">
+      <c r="C22" s="24" t="n">
         <v>9250</v>
       </c>
       <c r="D22" s="16" t="n">
@@ -1784,7 +1810,7 @@
           <t>COMISION MANTENIMIENTO</t>
         </is>
       </c>
-      <c r="C23" s="22" t="n">
+      <c r="C23" s="24" t="n">
         <v>4800</v>
       </c>
       <c r="D23" s="16" t="n">
@@ -1792,25 +1818,6 @@
       </c>
       <c r="E23" s="16">
         <f>E22+D23-C23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="17" t="inlineStr">
-        <is>
-          <t>TOTALES</t>
-        </is>
-      </c>
-      <c r="C24" s="16">
-        <f>SUM(C9:C23)</f>
-        <v/>
-      </c>
-      <c r="D24" s="16">
-        <f>SUM(D9:D23)</f>
-        <v/>
-      </c>
-      <c r="E24" s="16">
-        <f>E23</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Export FO 02-03: sin coincidencia siempre en verde (sin naranja por ahora)
</commit_message>
<xml_diff>
--- a/FO_02-03_DEMO.xlsx
+++ b/FO_02-03_DEMO.xlsx
@@ -10,7 +10,9 @@
     <sheet name="Libro Mayor" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Movimientos Bancarios" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Movimientos Bancarios'!$A$8:$E$24</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -64,7 +66,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -140,14 +142,11 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
-    <border>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -179,32 +178,35 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" shrinkToFit="1"/>
     </xf>
   </cellXfs>
@@ -572,16 +574,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
@@ -661,720 +663,446 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>Documento</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>Cuenta</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>Debe</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>Haber</t>
         </is>
       </c>
-      <c r="F8" s="15" t="inlineStr">
+      <c r="F9" s="15" t="inlineStr">
         <is>
           <t>Saldo</t>
         </is>
       </c>
-      <c r="G8" s="15" t="inlineStr">
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="H8" s="15" t="inlineStr">
+      <c r="H9" s="15" t="inlineStr">
         <is>
           <t>Organización</t>
         </is>
       </c>
-      <c r="I8" s="15" t="inlineStr">
+      <c r="I9" s="15" t="inlineStr">
         <is>
           <t>Centro de Costos</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="F9" s="16" t="n">
+    <row r="10">
+      <c r="A10" s="16" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Saldo Inicial</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="n"/>
+      <c r="D10" s="17" t="n"/>
+      <c r="E10" s="17" t="n"/>
+      <c r="F10" s="18" t="n">
         <v>1800000</v>
       </c>
-      <c r="G9" s="17" t="inlineStr">
-        <is>
-          <t>Saldo Inicial</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="18" t="n">
+      <c r="G10" s="17" t="n"/>
+      <c r="H10" s="17" t="n"/>
+      <c r="I10" s="17" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="n">
         <v>46204</v>
       </c>
-      <c r="B10" s="19" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>FCA-0001-00000001</t>
         </is>
       </c>
-      <c r="C10" s="19" t="inlineStr"/>
-      <c r="D10" s="20" t="n">
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" s="20" t="n">
         <v>1250000</v>
       </c>
-      <c r="E10" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="16">
-        <f>F9+D10-E10</f>
-        <v/>
-      </c>
-      <c r="G10" s="21" t="inlineStr">
+      <c r="F11" s="21">
+        <f>F10+D11-E11</f>
+        <v/>
+      </c>
+      <c r="G11" t="inlineStr">
         <is>
           <t>Factura A 1001 - Cliente Norte</t>
         </is>
       </c>
-      <c r="H10" s="21" t="inlineStr"/>
-      <c r="I10" s="21" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="18" t="n">
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="n">
         <v>46205</v>
       </c>
-      <c r="B11" s="19" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>REC-0002-00000001</t>
         </is>
       </c>
-      <c r="C11" s="19" t="inlineStr"/>
-      <c r="D11" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="20" t="n">
+      <c r="C12" t="inlineStr"/>
+      <c r="E12" s="20" t="n">
         <v>1250000</v>
       </c>
-      <c r="F11" s="16">
-        <f>F10+D11-E11</f>
-        <v/>
-      </c>
-      <c r="G11" s="21" t="inlineStr">
+      <c r="F12" s="21">
+        <f>F11+D12-E12</f>
+        <v/>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>Cobro factura A 1001</t>
         </is>
       </c>
-      <c r="H11" s="21" t="inlineStr"/>
-      <c r="I11" s="21" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="18" t="n">
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="n">
         <v>46206</v>
       </c>
-      <c r="B12" s="19" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>FCA-0001-00000002</t>
         </is>
       </c>
-      <c r="C12" s="19" t="inlineStr"/>
-      <c r="D12" s="20" t="n">
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" s="20" t="n">
         <v>845000.5</v>
       </c>
-      <c r="E12" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="16">
-        <f>F11+D12-E12</f>
-        <v/>
-      </c>
-      <c r="G12" s="21" t="inlineStr">
+      <c r="F13" s="21">
+        <f>F12+D13-E13</f>
+        <v/>
+      </c>
+      <c r="G13" t="inlineStr">
         <is>
           <t>Factura A 1002 - Cliente Sur</t>
         </is>
       </c>
-      <c r="H12" s="21" t="inlineStr"/>
-      <c r="I12" s="21" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="18" t="n">
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="n">
         <v>46207</v>
       </c>
-      <c r="B13" s="19" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>OP-0003-00000001</t>
         </is>
       </c>
-      <c r="C13" s="19" t="inlineStr"/>
-      <c r="D13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="20" t="n">
+      <c r="C14" t="inlineStr"/>
+      <c r="E14" s="20" t="n">
         <v>320000</v>
       </c>
-      <c r="F13" s="16">
-        <f>F12+D13-E13</f>
-        <v/>
-      </c>
-      <c r="G13" s="21" t="inlineStr">
+      <c r="F14" s="21">
+        <f>F13+D14-E14</f>
+        <v/>
+      </c>
+      <c r="G14" t="inlineStr">
         <is>
           <t>Pago proveedor Logistica SRL</t>
         </is>
       </c>
-      <c r="H13" s="21" t="inlineStr"/>
-      <c r="I13" s="21" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="18" t="n">
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="n">
         <v>46208</v>
       </c>
-      <c r="B14" s="19" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>OP-0003-00000002</t>
         </is>
       </c>
-      <c r="C14" s="19" t="inlineStr"/>
-      <c r="D14" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="20" t="n">
+      <c r="C15" t="inlineStr"/>
+      <c r="E15" s="20" t="n">
         <v>180000</v>
       </c>
-      <c r="F14" s="16">
-        <f>F13+D14-E14</f>
-        <v/>
-      </c>
-      <c r="G14" s="21" t="inlineStr">
+      <c r="F15" s="21">
+        <f>F14+D15-E15</f>
+        <v/>
+      </c>
+      <c r="G15" t="inlineStr">
         <is>
           <t>Honorarios contables</t>
         </is>
       </c>
-      <c r="H14" s="21" t="inlineStr"/>
-      <c r="I14" s="21" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="18" t="n">
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="n">
         <v>46211</v>
       </c>
-      <c r="B15" s="19" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>ASI-0004-00000001</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr"/>
-      <c r="D15" s="20" t="n">
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" s="20" t="n">
         <v>15500.75</v>
       </c>
-      <c r="E15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="16">
-        <f>F14+D15-E15</f>
-        <v/>
-      </c>
-      <c r="G15" s="21" t="inlineStr">
+      <c r="F16" s="21">
+        <f>F15+D16-E16</f>
+        <v/>
+      </c>
+      <c r="G16" t="inlineStr">
         <is>
           <t>Comisiones bancarias</t>
         </is>
       </c>
-      <c r="H15" s="21" t="inlineStr"/>
-      <c r="I15" s="21" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="18" t="n">
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="n">
         <v>46213</v>
       </c>
-      <c r="B16" s="19" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>FCA-0001-00000003</t>
         </is>
       </c>
-      <c r="C16" s="19" t="inlineStr"/>
-      <c r="D16" s="20" t="n">
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" s="20" t="n">
         <v>530000</v>
       </c>
-      <c r="E16" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="16">
-        <f>F15+D16-E16</f>
-        <v/>
-      </c>
-      <c r="G16" s="21" t="inlineStr">
+      <c r="F17" s="21">
+        <f>F16+D17-E17</f>
+        <v/>
+      </c>
+      <c r="G17" t="inlineStr">
         <is>
           <t>Factura A 1003 - Cliente Centro</t>
         </is>
       </c>
-      <c r="H16" s="21" t="inlineStr"/>
-      <c r="I16" s="21" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="18" t="n">
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="19" t="n">
         <v>46215</v>
       </c>
-      <c r="B17" s="19" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>OP-0003-00000003</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr"/>
-      <c r="D17" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="20" t="n">
+      <c r="C18" t="inlineStr"/>
+      <c r="E18" s="20" t="n">
         <v>96000</v>
       </c>
-      <c r="F17" s="16">
-        <f>F16+D17-E17</f>
-        <v/>
-      </c>
-      <c r="G17" s="21" t="inlineStr">
+      <c r="F18" s="21">
+        <f>F17+D18-E18</f>
+        <v/>
+      </c>
+      <c r="G18" t="inlineStr">
         <is>
           <t>Transferencia seguro</t>
         </is>
       </c>
-      <c r="H17" s="21" t="inlineStr"/>
-      <c r="I17" s="21" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="18" t="n">
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="n">
         <v>46218</v>
       </c>
-      <c r="B18" s="19" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>REC-0002-00000002</t>
         </is>
       </c>
-      <c r="C18" s="19" t="inlineStr"/>
-      <c r="D18" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="20" t="n">
+      <c r="C19" t="inlineStr"/>
+      <c r="E19" s="20" t="n">
         <v>845000.5</v>
       </c>
-      <c r="F18" s="16">
-        <f>F17+D18-E18</f>
-        <v/>
-      </c>
-      <c r="G18" s="21" t="inlineStr">
+      <c r="F19" s="21">
+        <f>F18+D19-E19</f>
+        <v/>
+      </c>
+      <c r="G19" t="inlineStr">
         <is>
           <t>Cobro factura A 1002</t>
         </is>
       </c>
-      <c r="H18" s="21" t="inlineStr"/>
-      <c r="I18" s="21" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="18" t="n">
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="19" t="n">
         <v>46221</v>
       </c>
-      <c r="B19" s="19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>FCA-0001-00000004</t>
         </is>
       </c>
-      <c r="C19" s="19" t="inlineStr"/>
-      <c r="D19" s="20" t="n">
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" s="20" t="n">
         <v>410000</v>
       </c>
-      <c r="E19" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="16">
-        <f>F18+D19-E19</f>
-        <v/>
-      </c>
-      <c r="G19" s="21" t="inlineStr">
+      <c r="F20" s="21">
+        <f>F19+D20-E20</f>
+        <v/>
+      </c>
+      <c r="G20" t="inlineStr">
         <is>
           <t>Factura A 1004 - Cliente Norte</t>
         </is>
       </c>
-      <c r="H19" s="21" t="inlineStr"/>
-      <c r="I19" s="21" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="18" t="n">
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="19" t="n">
         <v>46223</v>
       </c>
-      <c r="B20" s="19" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>OP-0003-00000004</t>
         </is>
       </c>
-      <c r="C20" s="19" t="inlineStr"/>
-      <c r="D20" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="20" t="n">
+      <c r="C21" t="inlineStr"/>
+      <c r="E21" s="20" t="n">
         <v>250000</v>
       </c>
-      <c r="F20" s="16">
-        <f>F19+D20-E20</f>
-        <v/>
-      </c>
-      <c r="G20" s="21" t="inlineStr">
+      <c r="F21" s="21">
+        <f>F20+D21-E21</f>
+        <v/>
+      </c>
+      <c r="G21" t="inlineStr">
         <is>
           <t>Pago alquiler oficina</t>
         </is>
       </c>
-      <c r="H20" s="21" t="inlineStr"/>
-      <c r="I20" s="21" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="18" t="n">
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="19" t="n">
         <v>46225</v>
       </c>
-      <c r="B21" s="19" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>ASI-0004-00000002</t>
         </is>
       </c>
-      <c r="C21" s="19" t="inlineStr"/>
-      <c r="D21" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="20" t="n">
+      <c r="C22" t="inlineStr"/>
+      <c r="E22" s="20" t="n">
         <v>3200.25</v>
       </c>
-      <c r="F21" s="16">
-        <f>F20+D21-E21</f>
-        <v/>
-      </c>
-      <c r="G21" s="21" t="inlineStr">
+      <c r="F22" s="21">
+        <f>F21+D22-E22</f>
+        <v/>
+      </c>
+      <c r="G22" t="inlineStr">
         <is>
           <t>Intereses ganados</t>
         </is>
       </c>
-      <c r="H21" s="21" t="inlineStr"/>
-      <c r="I21" s="21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="18" t="n">
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="n">
         <v>46228</v>
       </c>
-      <c r="B22" s="19" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>FCA-0001-00000005</t>
         </is>
       </c>
-      <c r="C22" s="19" t="inlineStr"/>
-      <c r="D22" s="20" t="n">
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" s="20" t="n">
         <v>275000</v>
       </c>
-      <c r="E22" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="16">
-        <f>F21+D22-E22</f>
-        <v/>
-      </c>
-      <c r="G22" s="21" t="inlineStr">
+      <c r="F23" s="21">
+        <f>F22+D23-E23</f>
+        <v/>
+      </c>
+      <c r="G23" t="inlineStr">
         <is>
           <t>Factura A 1005 - Cliente Sur</t>
         </is>
       </c>
-      <c r="H22" s="21" t="inlineStr"/>
-      <c r="I22" s="21" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="18" t="n">
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="n">
         <v>46231</v>
       </c>
-      <c r="B23" s="19" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>OP-0003-00000005</t>
         </is>
       </c>
-      <c r="C23" s="19" t="inlineStr"/>
-      <c r="D23" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="20" t="n">
+      <c r="C24" t="inlineStr"/>
+      <c r="E24" s="20" t="n">
         <v>198000</v>
       </c>
-      <c r="F23" s="16">
-        <f>F22+D23-E23</f>
-        <v/>
-      </c>
-      <c r="G23" s="21" t="inlineStr">
+      <c r="F24" s="21">
+        <f>F23+D24-E24</f>
+        <v/>
+      </c>
+      <c r="G24" t="inlineStr">
         <is>
           <t>Pago proveedor Insumos SA</t>
         </is>
       </c>
-      <c r="H23" s="21" t="inlineStr"/>
-      <c r="I23" s="21" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="18" t="n">
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="n">
         <v>46233</v>
       </c>
-      <c r="B24" s="19" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>REC-0002-00000003</t>
         </is>
       </c>
-      <c r="C24" s="19" t="inlineStr"/>
-      <c r="D24" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="16" t="n">
+      <c r="C25" t="inlineStr"/>
+      <c r="E25" s="22" t="n">
         <v>530000</v>
       </c>
-      <c r="F24" s="16">
-        <f>F23+D24-E24</f>
-        <v/>
-      </c>
-      <c r="G24" s="21" t="inlineStr">
+      <c r="F25" s="21">
+        <f>F24+D25-E25</f>
+        <v/>
+      </c>
+      <c r="G25" t="inlineStr">
         <is>
           <t>Cobro factura A 1003</t>
         </is>
       </c>
-      <c r="H24" s="21" t="inlineStr"/>
-      <c r="I24" s="21" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="17" t="inlineStr">
-        <is>
-          <t>Partidas contables no registradas en banco.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="15" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-      <c r="B27" s="15" t="inlineStr">
-        <is>
-          <t>Documento</t>
-        </is>
-      </c>
-      <c r="C27" s="15" t="inlineStr">
-        <is>
-          <t>Cuenta</t>
-        </is>
-      </c>
-      <c r="D27" s="15" t="inlineStr">
-        <is>
-          <t>Debe</t>
-        </is>
-      </c>
-      <c r="E27" s="15" t="inlineStr">
-        <is>
-          <t>Haber</t>
-        </is>
-      </c>
-      <c r="F27" s="15" t="inlineStr">
-        <is>
-          <t>Saldo</t>
-        </is>
-      </c>
-      <c r="G27" s="15" t="inlineStr">
-        <is>
-          <t>Descripción</t>
-        </is>
-      </c>
-      <c r="H27" s="15" t="inlineStr">
-        <is>
-          <t>Organización</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="18" t="n">
-        <v>46233</v>
-      </c>
-      <c r="B28" s="19" t="inlineStr">
-        <is>
-          <t>REC-0002-00000003</t>
-        </is>
-      </c>
-      <c r="C28" s="19" t="inlineStr"/>
-      <c r="D28" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="16" t="n">
-        <v>530000</v>
-      </c>
-      <c r="F28" s="16">
-        <f>D28-E28</f>
-        <v/>
-      </c>
-      <c r="G28" s="21" t="inlineStr">
-        <is>
-          <t>Cobro factura A 1003</t>
-        </is>
-      </c>
-      <c r="H28" s="21" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="18" t="n">
-        <v>46234</v>
-      </c>
-      <c r="B29" s="19" t="inlineStr">
-        <is>
-          <t>FCA-0001-00000006</t>
-        </is>
-      </c>
-      <c r="C29" s="19" t="inlineStr"/>
-      <c r="D29" s="16" t="n">
-        <v>620000</v>
-      </c>
-      <c r="E29" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" s="16">
-        <f>F28+D29-E29</f>
-        <v/>
-      </c>
-      <c r="G29" s="21" t="inlineStr">
-        <is>
-          <t>Factura A 1006 - pendiente de cobro</t>
-        </is>
-      </c>
-      <c r="H29" s="21" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="17" t="inlineStr">
-        <is>
-          <t>Partidas en banco pendientes de registración contable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="15" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-      <c r="B32" s="15" t="inlineStr">
-        <is>
-          <t>Documento</t>
-        </is>
-      </c>
-      <c r="C32" s="15" t="inlineStr">
-        <is>
-          <t>Cuenta</t>
-        </is>
-      </c>
-      <c r="D32" s="15" t="inlineStr">
-        <is>
-          <t>Debe</t>
-        </is>
-      </c>
-      <c r="E32" s="15" t="inlineStr">
-        <is>
-          <t>Haber</t>
-        </is>
-      </c>
-      <c r="F32" s="15" t="inlineStr">
-        <is>
-          <t>Saldo</t>
-        </is>
-      </c>
-      <c r="G32" s="15" t="inlineStr">
-        <is>
-          <t>Descripción</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="18" t="n">
-        <v>46234</v>
-      </c>
-      <c r="B33" s="19" t="inlineStr">
-        <is>
-          <t>IMP-0001</t>
-        </is>
-      </c>
-      <c r="C33" s="19" t="inlineStr"/>
-      <c r="D33" s="21" t="n"/>
-      <c r="E33" s="16" t="n">
-        <v>9250</v>
-      </c>
-      <c r="F33" s="16">
-        <f>F32+D33-E33</f>
-        <v/>
-      </c>
-      <c r="G33" s="21" t="inlineStr">
-        <is>
-          <t>IMPUESTO LEY 25413</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="18" t="n">
-        <v>46234</v>
-      </c>
-      <c r="B34" s="19" t="inlineStr">
-        <is>
-          <t>COM-0002</t>
-        </is>
-      </c>
-      <c r="C34" s="19" t="inlineStr"/>
-      <c r="D34" s="21" t="n"/>
-      <c r="E34" s="16" t="n">
-        <v>4800</v>
-      </c>
-      <c r="F34" s="16">
-        <f>F33+D34-E34</f>
-        <v/>
-      </c>
-      <c r="G34" s="21" t="inlineStr">
-        <is>
-          <t>COMISION MANTENIMIENTO</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="17" t="inlineStr">
-        <is>
-          <t>Total gastos e impuestos pendientes</t>
-        </is>
-      </c>
-      <c r="E35" s="16">
-        <f>SUM(E33:E34)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="17" t="inlineStr">
-        <is>
-          <t>Saldo Ajustado</t>
-        </is>
-      </c>
-      <c r="F37" s="16">
-        <f>F24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="17" t="inlineStr">
-        <is>
-          <t>Saldo según Extracto</t>
-        </is>
-      </c>
-      <c r="F38" s="16" t="n">
-        <v>2916950.75</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="17" t="inlineStr">
-        <is>
-          <t>Control de diferencia</t>
-        </is>
-      </c>
-      <c r="F39" s="16">
-        <f>F37-F38</f>
-        <v/>
-      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1391,16 +1119,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -1502,326 +1231,316 @@
           <t>Saldo en $</t>
         </is>
       </c>
-      <c r="G8" s="22" t="inlineStr">
-        <is>
-          <t>Total Débitos</t>
-        </is>
-      </c>
-      <c r="H8" s="23">
-        <f>SUM(C9:C23)</f>
-        <v/>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="J8" s="23" t="inlineStr">
+        <is>
+          <t>Suma Crédito</t>
+        </is>
+      </c>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>Suma Débito</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="n">
+      <c r="A9" s="17" t="n"/>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Saldo Inicial</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="n"/>
+      <c r="D9" s="17" t="n"/>
+      <c r="E9" s="18" t="n">
+        <v>2916950.75</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>IMPUESTO LEY 25413</t>
+        </is>
+      </c>
+      <c r="J9" s="24" t="n"/>
+      <c r="K9" s="24" t="n">
+        <v>9250</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="n">
         <v>46204</v>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>SALDO INICIAL</t>
         </is>
       </c>
-      <c r="C9" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="16">
-        <f>D9-C9</f>
-        <v/>
-      </c>
-      <c r="G9" s="22" t="inlineStr">
-        <is>
-          <t>Total Créditos</t>
-        </is>
-      </c>
-      <c r="H9" s="23">
-        <f>SUM(D9:D23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="18" t="n">
+      <c r="E10" s="21">
+        <f>E9+D10+C10</f>
+        <v/>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>COMISION MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="J10" s="24" t="n"/>
+      <c r="K10" s="24" t="n">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="n">
         <v>46205</v>
       </c>
-      <c r="B10" s="19" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>TRANSFERENCIA RECIBIDA CLIENTE NORTE</t>
         </is>
       </c>
-      <c r="C10" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="20" t="n">
+      <c r="D11" s="20" t="n">
         <v>1250000</v>
       </c>
-      <c r="E10" s="16">
-        <f>E9+D10-C10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="18" t="n">
+      <c r="E11" s="21">
+        <f>E10+D11+C11</f>
+        <v/>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="J11" s="25" t="n"/>
+      <c r="K11" s="25" t="n">
+        <v>14050</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="n">
         <v>46207</v>
       </c>
-      <c r="B11" s="19" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>PAGO PROVEEDOR LOGISTICA SRL</t>
         </is>
       </c>
-      <c r="C11" s="20" t="n">
-        <v>320000</v>
-      </c>
-      <c r="D11" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="16">
-        <f>E10+D11-C11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="18" t="n">
+      <c r="C12" s="20" t="n">
+        <v>-320000</v>
+      </c>
+      <c r="E12" s="21">
+        <f>E11+D12+C12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="n">
         <v>46210</v>
       </c>
-      <c r="B12" s="19" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>DEBITO AUTOMATICO EDESUR</t>
         </is>
       </c>
-      <c r="C12" s="20" t="n">
-        <v>48200</v>
-      </c>
-      <c r="D12" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="16">
-        <f>E11+D12-C12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="18" t="n">
+      <c r="C13" s="20" t="n">
+        <v>-48200</v>
+      </c>
+      <c r="E13" s="21">
+        <f>E12+D13+C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="n">
         <v>46213</v>
       </c>
-      <c r="B13" s="19" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>TRANSFERENCIA RECIBIDA CLIENTE CENTRO</t>
         </is>
       </c>
-      <c r="C13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="20" t="n">
+      <c r="D14" s="20" t="n">
         <v>530000</v>
       </c>
-      <c r="E13" s="16">
-        <f>E12+D13-C13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="18" t="n">
+      <c r="E14" s="21">
+        <f>E13+D14+C14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="n">
         <v>46215</v>
       </c>
-      <c r="B14" s="19" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>TRANSFERENCIA SEGURO</t>
         </is>
       </c>
-      <c r="C14" s="20" t="n">
-        <v>96000</v>
-      </c>
-      <c r="D14" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="16">
-        <f>E13+D14-C14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="18" t="n">
+      <c r="C15" s="20" t="n">
+        <v>-96000</v>
+      </c>
+      <c r="E15" s="21">
+        <f>E14+D15+C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="n">
         <v>46218</v>
       </c>
-      <c r="B15" s="19" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>TRANSFERENCIA RECIBIDA CLIENTE SUR</t>
         </is>
       </c>
-      <c r="C15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="20" t="n">
+      <c r="D16" s="20" t="n">
         <v>845000.5</v>
       </c>
-      <c r="E15" s="16">
-        <f>E14+D15-C15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="18" t="n">
+      <c r="E16" s="21">
+        <f>E15+D16+C16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="n">
         <v>46221</v>
       </c>
-      <c r="B16" s="19" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>DEPOSITO EFECTIVO</t>
         </is>
       </c>
-      <c r="C16" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="20" t="n">
+      <c r="D17" s="20" t="n">
         <v>410000</v>
       </c>
-      <c r="E16" s="16">
-        <f>E15+D16-C16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="18" t="n">
+      <c r="E17" s="21">
+        <f>E16+D17+C17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="19" t="n">
         <v>46223</v>
       </c>
-      <c r="B17" s="19" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>TRANSFERENCIA ALQUILER OFICINA</t>
         </is>
       </c>
-      <c r="C17" s="20" t="n">
-        <v>250000</v>
-      </c>
-      <c r="D17" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="16">
-        <f>E16+D17-C17</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="18" t="n">
+      <c r="C18" s="20" t="n">
+        <v>-250000</v>
+      </c>
+      <c r="E18" s="21">
+        <f>E17+D18+C18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="n">
         <v>46225</v>
       </c>
-      <c r="B18" s="19" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>ACREDITACION INTERESES</t>
         </is>
       </c>
-      <c r="C18" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="20" t="n">
+      <c r="D19" s="20" t="n">
         <v>3200.25</v>
       </c>
-      <c r="E18" s="16">
-        <f>E17+D18-C18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="18" t="n">
+      <c r="E19" s="21">
+        <f>E18+D19+C19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="19" t="n">
         <v>46228</v>
       </c>
-      <c r="B19" s="19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>TRANSFERENCIA RECIBIDA CLIENTE SUR</t>
         </is>
       </c>
-      <c r="C19" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="20" t="n">
+      <c r="D20" s="20" t="n">
         <v>275000</v>
       </c>
-      <c r="E19" s="16">
-        <f>E18+D19-C19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="18" t="n">
+      <c r="E20" s="21">
+        <f>E19+D20+C20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="19" t="n">
         <v>46231</v>
       </c>
-      <c r="B20" s="19" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>PAGO PROVEEDOR INSUMOS SA</t>
         </is>
       </c>
-      <c r="C20" s="20" t="n">
-        <v>198000</v>
-      </c>
-      <c r="D20" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="16">
-        <f>E19+D20-C20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="18" t="n">
+      <c r="C21" s="20" t="n">
+        <v>-198000</v>
+      </c>
+      <c r="E21" s="21">
+        <f>E20+D21+C21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="19" t="n">
         <v>46233</v>
       </c>
-      <c r="B21" s="19" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>TRANSFERENCIA RECIBIDA CLIENTE CENTRO</t>
         </is>
       </c>
-      <c r="C21" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="20" t="n">
+      <c r="D22" s="20" t="n">
         <v>530000</v>
       </c>
-      <c r="E21" s="16">
-        <f>E20+D21-C21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="18" t="n">
+      <c r="E22" s="21">
+        <f>E21+D22+C22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="n">
         <v>46234</v>
       </c>
-      <c r="B22" s="19" t="inlineStr">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>COMISION MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="n">
+        <v>-4800</v>
+      </c>
+      <c r="E23" s="21">
+        <f>E22+D23+C23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>IMPUESTO LEY 25413</t>
         </is>
       </c>
-      <c r="C22" s="24" t="n">
-        <v>9250</v>
-      </c>
-      <c r="D22" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="16">
-        <f>E21+D22-C22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="18" t="n">
-        <v>46234</v>
-      </c>
-      <c r="B23" s="19" t="inlineStr">
-        <is>
-          <t>COMISION MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="C23" s="24" t="n">
-        <v>4800</v>
-      </c>
-      <c r="D23" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="16">
-        <f>E22+D23-C23</f>
+      <c r="C24" s="22" t="n">
+        <v>-9250</v>
+      </c>
+      <c r="E24" s="21">
+        <f>E23+D24+C24</f>
         <v/>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A8:E24"/>
   <mergeCells count="2">
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="C2:H2"/>

</xml_diff>